<commit_message>
modified:   data/random_lat_lon_points.xlsx 	new file:   data/test.xlsx 	modified:   pv_console/config.py 	modified:   pv_console/streamlit_app.py
</commit_message>
<xml_diff>
--- a/data/random_lat_lon_points.xlsx
+++ b/data/random_lat_lon_points.xlsx
@@ -30,19 +30,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -78,18 +72,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -403,12 +391,12 @@
   <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -420,277 +408,277 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
-      <c r="A2" s="3">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
-        <v>28.6129</v>
-      </c>
-      <c r="C2" s="4">
-        <v>77.2295</v>
+      <c r="B2" s="2">
+        <v>18.535567</v>
+      </c>
+      <c r="C2" s="2">
+        <v>73.887565</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="3">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="4">
-        <v>18.55</v>
-      </c>
-      <c r="C3" s="4">
-        <v>73.93</v>
+      <c r="B3" s="2">
+        <v>18.54988</v>
+      </c>
+      <c r="C3" s="2">
+        <v>73.92594</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="3">
+      <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="4">
-        <v>13.0827</v>
-      </c>
-      <c r="C4" s="4">
-        <v>80.2707</v>
+      <c r="B4" s="2">
+        <v>18.54987</v>
+      </c>
+      <c r="C4" s="2">
+        <v>73.92609</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
-      <c r="A5" s="3">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="2">
         <v>22.5726</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="2">
         <v>88.3639</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="3">
+      <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="2">
         <v>23.0225</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="2">
         <v>72.5714</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="3">
+      <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="2">
         <v>15.2993</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="2">
         <v>74.124</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="3">
+      <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="2">
         <v>26.8467</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="2">
         <v>80.9462</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="3">
+      <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="2">
         <v>11.0168</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="2">
         <v>76.9558</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
-      <c r="A10" s="3">
+      <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="2">
         <v>21.1702</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="2">
         <v>72.8311</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
-      <c r="A11" s="3">
+      <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="2">
         <v>25.5941</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="2">
         <v>85.1376</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="3">
+      <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="2">
         <v>34.0522</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="2">
         <v>-118.2437</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
-      <c r="A13" s="3">
+      <c r="A13" s="1">
         <v>12</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="2">
         <v>40.7128</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="2">
         <v>-74.006</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="3">
+      <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="2">
         <v>51.5074</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C14" s="2">
         <v>-0.1278</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
-      <c r="A15" s="3">
+      <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="2">
         <v>-33.8688</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C15" s="2">
         <v>151.2093</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
-      <c r="A16" s="3">
+      <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="2">
         <v>35.6895</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="2">
         <v>139.6917</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
-      <c r="A17" s="3">
+      <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="2">
         <v>-23.5505</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="2">
         <v>-46.6333</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
-      <c r="A18" s="3">
+      <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="2">
         <v>55.7558</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="2">
         <v>37.6173</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="3">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
+      <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="2">
         <v>-1.2921</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="2">
         <v>36.8219</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="3">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
+      <c r="A20" s="1">
         <v>19</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="2">
         <v>52.3676</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C20" s="2">
         <v>4.9041</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="3">
+      <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B21" s="2">
         <v>-34.6037</v>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="2">
         <v>-58.3816</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="3">
+      <c r="A22" s="1">
         <v>21</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B22" s="2">
         <v>24.7536</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="2">
         <v>93.9023</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="3">
+      <c r="A23" s="1">
         <v>22</v>
       </c>
-      <c r="B23" s="4">
+      <c r="B23" s="2">
         <v>32.2265</v>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="2">
         <v>75.5433</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="3">
+      <c r="A24" s="1">
         <v>23</v>
       </c>
-      <c r="B24" s="4">
+      <c r="B24" s="2">
         <v>17.6868</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C24" s="2">
         <v>83.2185</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="3">
+      <c r="A25" s="1">
         <v>24</v>
       </c>
-      <c r="B25" s="4">
+      <c r="B25" s="2">
         <v>-17.7134</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="2">
         <v>178.065</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="3">
+      <c r="A26" s="1">
         <v>25</v>
       </c>
-      <c r="B26" s="4">
+      <c r="B26" s="2">
         <v>64.2008</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="2">
         <v>-149.4937</v>
       </c>
     </row>

</xml_diff>